<commit_message>
Replace assets/Sacha-slam.xlsx with updated file
</commit_message>
<xml_diff>
--- a/assets/Sacha-slam.xlsx
+++ b/assets/Sacha-slam.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rpous\Documents\portfolio\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523DA4EA-5694-4370-A040-FC6E81160E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8FE4C8-91DC-49C7-803E-B43741B590EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -170,6 +170,24 @@
   </si>
   <si>
     <t>Adresse URL du portfolio : https://sacha.portfolio.lyblics.com/</t>
+  </si>
+  <si>
+    <t>SIO 2 - Cybersécurité : sécurisation des accès et des services, gestion
+des habilitations, durcissement, sauvegardes et continuité, analyse et
+remédiation de vulnérabilités.</t>
+  </si>
+  <si>
+    <t>SIO 2 - Développement en PHP orienté objet : conception et réalisation
+d'une application web (POO, architecture MVC, accès base de données),
+tests et mise en service.</t>
+  </si>
+  <si>
+    <t>Support et assistance aux utilisateurs : traitement des incidents et
+demandes, gestion des habilitations et du parc informatique,
+accompagnement des utilisateurs et rédaction de procédures.</t>
+  </si>
+  <si>
+    <t>deploiment de l'application permettant de gérer les données et les tickets</t>
   </si>
 </sst>
 </file>
@@ -718,15 +736,39 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -758,30 +800,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1158,56 +1176,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="26"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="44" t="s">
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="39"/>
-      <c r="H3" s="45"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="32"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="43"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1219,22 +1237,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="41" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1257,8 +1275,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25"/>
-      <c r="B7" s="34"/>
+      <c r="A7" s="34"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1314,16 +1332,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1750,14 +1768,18 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="55.2" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
       <c r="E17" s="17"/>
       <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
+      <c r="G17" s="22"/>
       <c r="H17" s="18"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1795,14 +1817,18 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11"/>
-      <c r="B18" s="10"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="69" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>30</v>
+      </c>
       <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
+      <c r="D18" s="22"/>
       <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
       <c r="H18" s="18"/>
       <c r="I18"/>
       <c r="J18"/>
@@ -1931,16 +1957,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="32"/>
+      <c r="B21" s="39"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="40"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1977,14 +2003,18 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
       <c r="E22" s="17"/>
       <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
+      <c r="G22" s="22"/>
       <c r="H22" s="18"/>
       <c r="I22"/>
       <c r="J22"/>
@@ -2293,16 +2323,16 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A29" s="30" t="s">
+      <c r="A29" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="32"/>
+      <c r="B29" s="39"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="40"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2350,7 +2380,7 @@
       <c r="D30" s="22"/>
       <c r="E30" s="22"/>
       <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
+      <c r="G30" s="17"/>
       <c r="H30" s="22"/>
       <c r="I30"/>
       <c r="J30"/>
@@ -2389,14 +2419,18 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="11"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="17"/>
+      <c r="A31" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="22"/>
       <c r="D31" s="17"/>
       <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="18"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2751,11 +2785,6 @@
     <row r="83" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2763,6 +2792,11 @@
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>